<commit_message>
Meghívottak kijelölése: a helyszínhez közel lakók előre
- Tagoknál irányítószám + lakóhely (település), az importsablonban is; pontos utcacím nem kell
- Koordináta az OpenStreetMap Nominatim szolgáltatással a háttérben (1 kérés/mp, gyorsítótár,
  hálózati hiba után újrapróbálás); GEOCODING=off kikapcsolja
- Meghívottválasztó: szólamon belül légvonalbeli távolság szerint rendezve, km kijelzéssel;
  lakóhely nélküliek a szólam végén
- Tesztek, demóadatok, README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqK5QRU9YGqtKeGywQEwCy
</commit_message>
<xml_diff>
--- a/templates/tagok_import_sablon.xlsx
+++ b/templates/tagok_import_sablon.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>Vezetéknév</t>
   </si>
@@ -29,6 +29,12 @@
     <t>Szólam</t>
   </si>
   <si>
+    <t>Irányítószám</t>
+  </si>
+  <si>
+    <t>Lakóhely (település)</t>
+  </si>
+  <si>
     <t>Cantemus Vegyeskar</t>
   </si>
   <si>
@@ -53,6 +59,12 @@
     <t>Szoprán 1</t>
   </si>
   <si>
+    <t>4400</t>
+  </si>
+  <si>
+    <t>Nyíregyháza</t>
+  </si>
+  <si>
     <t>igen</t>
   </si>
   <si>
@@ -74,6 +86,12 @@
     <t>Basszus 2</t>
   </si>
   <si>
+    <t>4300</t>
+  </si>
+  <si>
+    <t>Nyírbátor</t>
+  </si>
+  <si>
     <t>Szabó</t>
   </si>
   <si>
@@ -102,6 +120,9 @@
   </si>
   <si>
     <t>Szólam: szabad szöveg, pl. Szoprán 1, Alt 2, Tenor 1, Basszus 2.</t>
+  </si>
+  <si>
+    <t>Irányítószám és Lakóhely (település): nem kötelező. Ebből számolja az app, ki lakik közel egy esemény helyszínéhez (pontos utcacímet nem kérünk).</t>
   </si>
   <si>
     <t>Admin: „igen”, ha a tag kezelheti az eseményeket és a tagokat.</t>
@@ -502,19 +523,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" style="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" customWidth="1"/>
     <col min="4" max="4" width="18" style="1" customWidth="1"/>
     <col min="5" max="5" width="14" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13" style="1" customWidth="1"/>
+    <col min="7" max="7" width="22" style="1" customWidth="1"/>
+    <col min="8" max="8" width="20" style="1" customWidth="1"/>
+    <col min="9" max="9" width="14" style="1" customWidth="1"/>
+    <col min="10" max="10" width="10" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -539,83 +562,107 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="I3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -626,7 +673,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -634,37 +681,42 @@
   <sheetData>
     <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Kisegítő művészek: harmadik tagi kategória, egyenkénti meghívás és naptárba mentés
- Új tagi jelölés (members.is_guest): külsős kisegítő, kórus nélkül; tagimport „Kisegítő művész” oszlop.
- Eseményenként egyenként meghívhatók (event_guests); csak a meghívott eseményeiket látják,
  csak azokról kapnak értesítést, emlékeztetőt; a riportban „Kisegítő művész”-ként szerepelnek.
- Esemény oldalán „Mentés a naptárba”: .ics (titkos naptárkulccsal, bejelentkezés nélkül) és Google Naptár link.
- Admin: kategória szűrő és jelölés a tagoknál, kisegítő-választó az eseményűrlapon.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqK5QRU9YGqtKeGywQEwCy
</commit_message>
<xml_diff>
--- a/templates/tagok_import_sablon.xlsx
+++ b/templates/tagok_import_sablon.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="48">
   <si>
     <t>Vezetéknév</t>
   </si>
@@ -41,6 +41,9 @@
     <t>Pro Musica</t>
   </si>
   <si>
+    <t>Kisegítő művész</t>
+  </si>
+  <si>
     <t>Admin</t>
   </si>
   <si>
@@ -107,6 +110,27 @@
     <t>Alt 1</t>
   </si>
   <si>
+    <t>Tóth</t>
+  </si>
+  <si>
+    <t>Gábor</t>
+  </si>
+  <si>
+    <t>toth.gabor@example.com</t>
+  </si>
+  <si>
+    <t>+36 70 111 2222</t>
+  </si>
+  <si>
+    <t>Tenor</t>
+  </si>
+  <si>
+    <t>4025</t>
+  </si>
+  <si>
+    <t>Debrecen</t>
+  </si>
+  <si>
     <t>Kitöltési útmutató</t>
   </si>
   <si>
@@ -119,7 +143,10 @@
     <t>Cantemus Vegyeskar / Pro Musica: „igen” vagy „nem”. Aki mindkettőnek tagja, mindkettőhöz „igen”-t írj.</t>
   </si>
   <si>
-    <t>Szólam: szabad szöveg, pl. Szoprán 1, Alt 2, Tenor 1, Basszus 2.</t>
+    <t>Kisegítő művész: „igen”, ha külsős (nem kórustag). Ő nem kap meghívást a kórus eseményeire, csak azokra, amelyekre az eseménynél egyenként kijelölöd; az eseményeket egyenként mentheti a naptárába. Kisegítő művésznél a kórusoszlopokat hagyd „nem”-en.</t>
+  </si>
+  <si>
+    <t>Szólam: szabad szöveg, pl. Szoprán 1, Alt 2, Tenor 1, Basszus 2 (kisegítőnél akár hangszer is).</t>
   </si>
   <si>
     <t>Irányítószám és Lakóhely (település): nem kötelező. Ebből számolja az app, ki lakik közel egy esemény helyszínéhez (pontos utcacímet nem kérünk).</t>
@@ -523,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" style="1" customWidth="1"/>
@@ -534,10 +561,11 @@
     <col min="7" max="7" width="22" style="1" customWidth="1"/>
     <col min="8" max="8" width="20" style="1" customWidth="1"/>
     <col min="9" max="9" width="14" style="1" customWidth="1"/>
-    <col min="10" max="10" width="10" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17" style="1" customWidth="1"/>
+    <col min="11" max="11" width="10" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -568,101 +596,148 @@
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="J3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="H4" s="1" t="s">
+      <c r="J4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>18</v>
+      <c r="K5" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -673,7 +748,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -681,42 +756,47 @@
   <sheetData>
     <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>38</v>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>